<commit_message>
tmp: PC import file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2GtXu9LN9coxaEYEbURSb
</commit_message>
<xml_diff>
--- a/tmp/fix_upload3.xlsx
+++ b/tmp/fix_upload3.xlsx
@@ -894,7 +894,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;strong&gt;Аккумуляторный шуруповерт с насадками 5 в 1 (36 В, 6 Ач)&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;Многофункциональный аккумуляторный набор 5в1 – это универсальный комплект для любых работ: от сверления до резки и демонтажа. В основе — шуруповерт с набором сменных насадок, которые превращают его в пыль, перфоратор, гайковерт и болгарку. Один инструмент – максимум возможностей.&lt;/p&gt;&lt;h3&gt;Основные преимущества&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;5 инструментов в одном комплекте&lt;/li&gt;&lt;li&gt;Мощная аккумуляторная система 36V, 6Ah&lt;/li&gt;&lt;li&gt;Быстрое изменение насадок под разные задачи&lt;/li&gt;&lt;li&gt;Высокая производительность и универсальность&lt;/li&gt;&lt;li&gt;Компактность – замена целого набора инструментов&lt;/li&gt;&lt;li&gt;Экономия места и денег&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Где используется&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Строительство и ремонт&lt;/li&gt;&lt;li&gt;Монтажные работы&lt;/li&gt;&lt;li&gt;Работа с металлом, деревом и бетоном&lt;/li&gt;&lt;li&gt;СТО и гараж&lt;/li&gt;&lt;li&gt;Домашние мастерские&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Почему следует выбрать Набор 5в1 АКБ &lt;/h3&gt;&lt;p&gt;Этот комплект — один из самых универсальных на рынке. Вы получаете шуруповерт, мини-пилу, перфоратор, гайковерт и УШМ в одном устройстве. Благодаря сменным насадкам инструмент легко адаптируется под любую задачу, что делает его особенно удобным для мобильной работы.&lt;/p&gt;&lt;h3&gt;Технические характеристики&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Тип: аккумуляторный набор 5в1&lt;/li&gt;&lt;li&gt;Напряжение: 36V&lt;/li&gt;&lt;li&gt;Емкость АКБ: 6Ah&lt;/li&gt;&lt;li&gt;Тип аккумулятора: Li-Ion&lt;/li&gt;&lt;li&gt;Базовый инструмент: шуруповерт &lt;/li&gt;&lt;li&gt;Крутящий момент: до ~42 Нм&lt;/li&gt;&lt;li&gt;Скорость: 0–400 / 0–1300 об/мин&lt;/li&gt;&lt;li&gt;Ударный режим: есть&lt;/li&gt;&lt;li&gt;Насадки&lt;/li&gt;&lt;li&gt;Шуруповерт&lt;/li&gt;&lt;li&gt;Мини-пила (шина ~10 см)&lt;/li&gt;&lt;li&gt;Перфоратор (~1.6 Дж)&lt;/li&gt;&lt;li&gt;Гайковерт&lt;/li&gt;&lt;li&gt;Болгарка (диск до 125 мм)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Идеально подходит для&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Мастеров универсалов&lt;/li&gt;&lt;li&gt;Строителей&lt;/li&gt;&lt;li&gt;Автомехаников&lt;/li&gt;&lt;li&gt;Домашних мастеров&lt;/li&gt;&lt;li&gt;Выездных работ&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Комплектация&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Шуруповерт &lt;/li&gt;&lt;li&gt;Насадка-пила&lt;/li&gt;&lt;li&gt;Насадка-перфоратор&lt;/li&gt;&lt;li&gt;Насадка-гайковерт&lt;/li&gt;&lt;li&gt;Насадка-болгарка&lt;/li&gt;&lt;li&gt;Аккумулятор 36V 6Ah - 2 шт&lt;/li&gt;&lt;li&gt;Зарядное устройство&lt;/li&gt;&lt;li&gt;Инструкция&lt;/li&gt;&lt;li&gt;Кейс&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;&lt;strong&gt;Аккумуляторный шуруповерт с насадками 5 в 1 (36 В, 6 Ач)&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;Многофункциональный аккумуляторный набор 5в1 – это универсальный комплект для любых работ: от сверления до резки и демонтажа. В основе — шуруповерт с набором сменных насадок, которые превращают его в пилу, перфоратор, гайковерт и болгарку. Один инструмент – максимум возможностей.&lt;/p&gt;&lt;h3&gt;Основные преимущества&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;5 инструментов в одном комплекте&lt;/li&gt;&lt;li&gt;Мощная аккумуляторная система 36V, 6Ah&lt;/li&gt;&lt;li&gt;Быстрое изменение насадок под разные задачи&lt;/li&gt;&lt;li&gt;Высокая производительность и универсальность&lt;/li&gt;&lt;li&gt;Компактность – замена целого набора инструментов&lt;/li&gt;&lt;li&gt;Экономия места и денег&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Где используется&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Строительство и ремонт&lt;/li&gt;&lt;li&gt;Монтажные работы&lt;/li&gt;&lt;li&gt;Работа с металлом, деревом и бетоном&lt;/li&gt;&lt;li&gt;СТО и гараж&lt;/li&gt;&lt;li&gt;Домашние мастерские&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Почему следует выбрать Набор 5в1 АКБ &lt;/h3&gt;&lt;p&gt;Этот комплект — один из самых универсальных на рынке. Вы получаете шуруповерт, мини-пилу, перфоратор, гайковерт и УШМ в одном устройстве. Благодаря сменным насадкам инструмент легко адаптируется под любую задачу, что делает его особенно удобным для мобильной работы.&lt;/p&gt;&lt;h3&gt;Технические характеристики&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Тип: аккумуляторный набор 5в1&lt;/li&gt;&lt;li&gt;Напряжение: 36V&lt;/li&gt;&lt;li&gt;Емкость АКБ: 6Ah&lt;/li&gt;&lt;li&gt;Тип аккумулятора: Li-Ion&lt;/li&gt;&lt;li&gt;Базовый инструмент: шуруповерт &lt;/li&gt;&lt;li&gt;Крутящий момент: до ~42 Нм&lt;/li&gt;&lt;li&gt;Скорость: 0–400 / 0–1300 об/мин&lt;/li&gt;&lt;li&gt;Ударный режим: есть&lt;/li&gt;&lt;li&gt;Насадки&lt;/li&gt;&lt;li&gt;Шуруповерт&lt;/li&gt;&lt;li&gt;Мини-пила (шина ~10 см)&lt;/li&gt;&lt;li&gt;Перфоратор (~1.6 Дж)&lt;/li&gt;&lt;li&gt;Гайковерт&lt;/li&gt;&lt;li&gt;Болгарка (диск до 125 мм)&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Идеально подходит для&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Мастеров универсалов&lt;/li&gt;&lt;li&gt;Строителей&lt;/li&gt;&lt;li&gt;Автомехаников&lt;/li&gt;&lt;li&gt;Домашних мастеров&lt;/li&gt;&lt;li&gt;Выездных работ&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Комплектация&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Шуруповерт &lt;/li&gt;&lt;li&gt;Насадка-пила&lt;/li&gt;&lt;li&gt;Насадка-перфоратор&lt;/li&gt;&lt;li&gt;Насадка-гайковерт&lt;/li&gt;&lt;li&gt;Насадка-болгарка&lt;/li&gt;&lt;li&gt;Аккумулятор 36V 6Ah - 2 шт&lt;/li&gt;&lt;li&gt;Зарядное устройство&lt;/li&gt;&lt;li&gt;Инструкция&lt;/li&gt;&lt;li&gt;Кейс&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;strong&gt;Набор аккумуляторного инструмента 6 в 1 (36 В, 6 Ач)&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;Универсальный аккумуляторный набор 6в1 – это многофункциональный инструмент нового поколения. Одно базовое устройство с сменными насадками заменяет сразу шесть отдельных инструментов: шуруповерт, перфоратор, гайковерт, болгарку, пыль и даже мойку. Максимальная мобильность и функциональность в одном кейсе.&lt;/p&gt;&lt;h3&gt;Основные преимущества&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;6 инструментов в одном комплекте&lt;/li&gt;&lt;li&gt;Мощный аккумулятор 36V, 6Ah&lt;/li&gt;&lt;li&gt;Быстрая смена насадок&lt;/li&gt;&lt;li&gt;Компактность и мобильность&lt;/li&gt;&lt;li&gt;Универсальность для разных материалов&lt;/li&gt;&lt;li&gt;Экономия места и бюджета&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Где используется&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Строительство и ремонт&lt;/li&gt;&lt;li&gt;Монтажные работы&lt;/li&gt;&lt;li&gt;Работа с бетоном, металлом и деревом&lt;/li&gt;&lt;li&gt;СТО и гараж&lt;/li&gt;&lt;li&gt;Бытовые и хозяйственные задачи&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Почему следует выбрать Набор 6в1 АКБ &lt;/h3&gt;&lt;p&gt;Этот комплект позволяет выполнять полный спектр работ&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Шуруповерт – базовый инструмент для монтажа.&lt;/li&gt;&lt;li&gt;Перфоратор – сила удара ~1.4 Дж для бетона&lt;/li&gt;&lt;li&gt;Гайковерт - для работы с крепежами.&lt;/li&gt;&lt;li&gt;Болгарка – диск до 125 мм для резки&lt;/li&gt;&lt;li&gt;Мини-пила – шина ~10 см, скорость ~8 м/с&lt;/li&gt;&lt;li&gt;Мойка – для очистки поверхностей и техники&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Фактически это “инструмент-комбайн”, заменяющий полноценный набор оборудования.&lt;/p&gt;&lt;h3&gt;Технические характеристики&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Тип: аккумуляторный набор 6в1&lt;/li&gt;&lt;li&gt;Напряжение: 36V&lt;/li&gt;&lt;li&gt;Емкость АКБ: 6Ah&lt;/li&gt;&lt;li&gt;Тип аккумулятора: Li-Ion&lt;/li&gt;&lt;li&gt;Крутящий момент: до ~24 Нм&lt;/li&gt;&lt;li&gt;Скорость: 0–600 / 0–1800 об/мин&lt;/li&gt;&lt;li&gt;Перфоратор: до 5200 уд/мин, ~1.4 Дж&lt;/li&gt;&lt;li&gt;Болгарка: диск 125 мм&lt;/li&gt;&lt;li&gt;Пила: скорость цепи ~8 м/с&lt;/li&gt;&lt;li&gt;Вес комплекта: ~8 кг&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Идеально подходит для&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Мастеров универсалов&lt;/li&gt;&lt;li&gt;Строителей&lt;/li&gt;&lt;li&gt;Выездных работ&lt;/li&gt;&lt;li&gt;Домашних мастеров&lt;/li&gt;&lt;li&gt;Тех, кто хочет &amp;quot;все в одном&amp;quot;&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Комплектация&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Базовый инструмент &lt;/li&gt;&lt;li&gt;Насадка-шуруповерт&lt;/li&gt;&lt;li&gt;Насадка-перфоратор&lt;/li&gt;&lt;li&gt;Насадка-гайковерт&lt;/li&gt;&lt;li&gt;Насадка-болгарка&lt;/li&gt;&lt;li&gt;Насадка-пила&lt;/li&gt;&lt;li&gt;Насадка-мойка&lt;/li&gt;&lt;li&gt;Аккумулятор 6Ah - 2 шт&lt;/li&gt;&lt;li&gt;Зарядное устройство&lt;/li&gt;&lt;li&gt;Шланг, фильтр, аксессуары для мойки&lt;/li&gt;&lt;li&gt;Инструкция&lt;/li&gt;&lt;li&gt;Кейс&lt;/li&gt;&lt;/ul&gt;</t>
+          <t>&lt;p&gt;&lt;strong&gt;Набор аккумуляторного инструмента 6 в 1 (36 В, 6 Ач)&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;Универсальный аккумуляторный набор 6в1 – это многофункциональный инструмент нового поколения. Одно базовое устройство с сменными насадками заменяет сразу шесть отдельных инструментов: шуруповерт, перфоратор, гайковерт, болгарку, пилу и даже мойку. Максимальная мобильность и функциональность в одном кейсе.&lt;/p&gt;&lt;h3&gt;Основные преимущества&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;6 инструментов в одном комплекте&lt;/li&gt;&lt;li&gt;Мощный аккумулятор 36V, 6Ah&lt;/li&gt;&lt;li&gt;Быстрая смена насадок&lt;/li&gt;&lt;li&gt;Компактность и мобильность&lt;/li&gt;&lt;li&gt;Универсальность для разных материалов&lt;/li&gt;&lt;li&gt;Экономия места и бюджета&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Где используется&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Строительство и ремонт&lt;/li&gt;&lt;li&gt;Монтажные работы&lt;/li&gt;&lt;li&gt;Работа с бетоном, металлом и деревом&lt;/li&gt;&lt;li&gt;СТО и гараж&lt;/li&gt;&lt;li&gt;Бытовые и хозяйственные задачи&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Почему следует выбрать Набор 6в1 АКБ &lt;/h3&gt;&lt;p&gt;Этот комплект позволяет выполнять полный спектр работ&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Шуруповерт – базовый инструмент для монтажа.&lt;/li&gt;&lt;li&gt;Перфоратор – сила удара ~1.4 Дж для бетона&lt;/li&gt;&lt;li&gt;Гайковерт - для работы с крепежами.&lt;/li&gt;&lt;li&gt;Болгарка – диск до 125 мм для резки&lt;/li&gt;&lt;li&gt;Мини-пила – шина ~10 см, скорость ~8 м/с&lt;/li&gt;&lt;li&gt;Мойка – для очистки поверхностей и техники&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Фактически это “инструмент-комбайн”, заменяющий полноценный набор оборудования.&lt;/p&gt;&lt;h3&gt;Технические характеристики&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Тип: аккумуляторный набор 6в1&lt;/li&gt;&lt;li&gt;Напряжение: 36V&lt;/li&gt;&lt;li&gt;Емкость АКБ: 6Ah&lt;/li&gt;&lt;li&gt;Тип аккумулятора: Li-Ion&lt;/li&gt;&lt;li&gt;Крутящий момент: до ~24 Нм&lt;/li&gt;&lt;li&gt;Скорость: 0–600 / 0–1800 об/мин&lt;/li&gt;&lt;li&gt;Перфоратор: до 5200 уд/мин, ~1.4 Дж&lt;/li&gt;&lt;li&gt;Болгарка: диск 125 мм&lt;/li&gt;&lt;li&gt;Пила: скорость цепи ~8 м/с&lt;/li&gt;&lt;li&gt;Вес комплекта: ~8 кг&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Идеально подходит для&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Мастеров универсалов&lt;/li&gt;&lt;li&gt;Строителей&lt;/li&gt;&lt;li&gt;Выездных работ&lt;/li&gt;&lt;li&gt;Домашних мастеров&lt;/li&gt;&lt;li&gt;Тех, кто хочет &amp;quot;все в одном&amp;quot;&lt;/li&gt;&lt;/ul&gt;&lt;h3&gt;Комплектация&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;Базовый инструмент &lt;/li&gt;&lt;li&gt;Насадка-шуруповерт&lt;/li&gt;&lt;li&gt;Насадка-перфоратор&lt;/li&gt;&lt;li&gt;Насадка-гайковерт&lt;/li&gt;&lt;li&gt;Насадка-болгарка&lt;/li&gt;&lt;li&gt;Насадка-пила&lt;/li&gt;&lt;li&gt;Насадка-мойка&lt;/li&gt;&lt;li&gt;Аккумулятор 6Ah - 2 шт&lt;/li&gt;&lt;li&gt;Зарядное устройство&lt;/li&gt;&lt;li&gt;Шланг, фильтр, аксессуары для мойки&lt;/li&gt;&lt;li&gt;Инструкция&lt;/li&gt;&lt;li&gt;Кейс&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">

</xml_diff>